<commit_message>
Add in num_engine parameter and calcProp for the planeObj to correct super hornet data
</commit_message>
<xml_diff>
--- a/Sizing/engine_lookup.xlsx
+++ b/Sizing/engine_lookup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58BC38FA-D9F8-4FB1-8E93-3A77B6717EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A4EBEE0-5296-4C66-AA45-DACDED97F8C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37230" yWindow="-2340" windowWidth="17470" windowHeight="15410" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-5830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Engine Name</t>
   </si>
@@ -55,6 +55,9 @@
   </si>
   <si>
     <t>F135</t>
+  </si>
+  <si>
+    <t>F414</t>
   </si>
 </sst>
 </file>
@@ -373,7 +376,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" customWidth="1"/>
@@ -459,6 +462,32 @@
         <v>45000000</v>
       </c>
     </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>57800</v>
+      </c>
+      <c r="C4">
+        <v>97900</v>
+      </c>
+      <c r="D4">
+        <v>30</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>0.25</v>
+      </c>
+      <c r="G4">
+        <v>1700</v>
+      </c>
+      <c r="H4" s="1">
+        <v>45000000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated with three other engines: 11.9.25
</commit_message>
<xml_diff>
--- a/Sizing/engine_lookup.xlsx
+++ b/Sizing/engine_lookup.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevke\OneDrive\Documents\GitSeniorDesign\team10aiaa\Sizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A4EBEE0-5296-4C66-AA45-DACDED97F8C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4757973A-6C34-48F6-B901-7A27B200B089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-5830" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Engine Name</t>
   </si>
@@ -58,6 +58,12 @@
   </si>
   <si>
     <t>F414</t>
+  </si>
+  <si>
+    <t>F100</t>
+  </si>
+  <si>
+    <t>F110</t>
   </si>
 </sst>
 </file>
@@ -376,7 +382,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" customWidth="1"/>
@@ -488,6 +494,58 @@
         <v>45000000</v>
       </c>
     </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>79100</v>
+      </c>
+      <c r="C5">
+        <v>129600</v>
+      </c>
+      <c r="D5">
+        <v>32</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>0.35</v>
+      </c>
+      <c r="G5">
+        <v>1700</v>
+      </c>
+      <c r="H5" s="1">
+        <v>45000000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>84500</v>
+      </c>
+      <c r="C6">
+        <v>144600</v>
+      </c>
+      <c r="D6">
+        <v>30.4</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>0.61</v>
+      </c>
+      <c r="G6">
+        <v>1700</v>
+      </c>
+      <c r="H6" s="1">
+        <v>45000000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Quite a few changes -Changed wing defenition to be based on LE, cr, ct, span instead of sweeps and taper ratio -Cleaned up testPlanEval to become f18comparison -Deveoped a way of passing in an array of store names and getting weights, cd0, and fuel storage back with a new lookup table -Pulled mission sets out of the plane obj to be standalone and only passed in as function input
</commit_message>
<xml_diff>
--- a/Sizing/engine_lookup.xlsx
+++ b/Sizing/engine_lookup.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevke\OneDrive\Documents\GitSeniorDesign\team10aiaa\Sizing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4757973A-6C34-48F6-B901-7A27B200B089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E359E5-B52A-4C30-BE12-A40CDC346F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,30 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
-    <t>Engine Name</t>
-  </si>
-  <si>
-    <t>Sealevel Max Thrust (no AB)</t>
-  </si>
-  <si>
-    <t>Sealevel Max Thrust (AB)</t>
-  </si>
-  <si>
-    <t>Compressor PRC</t>
-  </si>
-  <si>
-    <t>Fan PRC</t>
-  </si>
-  <si>
-    <t>Bypass Ratio</t>
-  </si>
-  <si>
-    <t>T04 - Burner Outlet Temp (K)</t>
-  </si>
-  <si>
-    <t>QR - Lower Heating Value (J/kg)</t>
-  </si>
-  <si>
     <t>F404</t>
   </si>
   <si>
@@ -64,6 +40,30 @@
   </si>
   <si>
     <t>F110</t>
+  </si>
+  <si>
+    <t>engine_name</t>
+  </si>
+  <si>
+    <t>h0_maxThrust_AB</t>
+  </si>
+  <si>
+    <t>prc_compressor</t>
+  </si>
+  <si>
+    <t>prc_fan</t>
+  </si>
+  <si>
+    <t>bypass_ratio</t>
+  </si>
+  <si>
+    <t>T04</t>
+  </si>
+  <si>
+    <t>QR</t>
+  </si>
+  <si>
+    <t>h0_maxThrust_NoAB</t>
   </si>
 </sst>
 </file>
@@ -392,33 +392,33 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="B2">
         <v>48900</v>
@@ -444,7 +444,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B3">
         <v>125000</v>
@@ -470,7 +470,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B4">
         <v>57800</v>
@@ -496,7 +496,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B5">
         <v>79100</v>
@@ -522,7 +522,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B6">
         <v>84500</v>

</xml_diff>

<commit_message>
Added in function to get Raymer regression coefficents so I could put in MW aircraft. Athough their predictions are way off. Made an actual readme which is a todo list
</commit_message>
<xml_diff>
--- a/Sizing/engine_lookup.xlsx
+++ b/Sizing/engine_lookup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfile\Documents\MyDocuments\CODING\GitWorkingDirectory\team10aiaa\Sizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E359E5-B52A-4C30-BE12-A40CDC346F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01E765BE-F16D-4522-8316-3648A523C18A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>F404</t>
   </si>
@@ -64,6 +64,9 @@
   </si>
   <si>
     <t>h0_maxThrust_NoAB</t>
+  </si>
+  <si>
+    <t>H20</t>
   </si>
 </sst>
 </file>
@@ -382,7 +385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" customWidth="1"/>
@@ -546,6 +549,32 @@
         <v>45000000</v>
       </c>
     </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>220</v>
+      </c>
+      <c r="C7">
+        <v>480</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>0.1</v>
+      </c>
+      <c r="G7">
+        <v>1700</v>
+      </c>
+      <c r="H7" s="1">
+        <v>45000000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>